<commit_message>
refactored code + improved upload and export feature
</commit_message>
<xml_diff>
--- a/data/sample.xlsx
+++ b/data/sample.xlsx
@@ -429,499 +429,1344 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>product_sku_code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>yearweek</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>nielsen_total_volume</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B2" s="2" t="n">
         <v>44562</v>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>23432</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B3" s="2" t="n">
         <v>44563</v>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
         <v>28964</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B4" s="2" t="n">
         <v>44564</v>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>30589</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B5" s="2" t="n">
         <v>44565</v>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>19264</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B6" s="2" t="n">
         <v>44566</v>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>13131</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B7" s="2" t="n">
         <v>44567</v>
       </c>
-      <c r="B7" t="n">
+      <c r="C7" t="n">
         <v>13443</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B8" s="2" t="n">
         <v>44568</v>
       </c>
-      <c r="B8" t="n">
+      <c r="C8" t="n">
         <v>23149</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B9" s="2" t="n">
         <v>44569</v>
       </c>
-      <c r="B9" t="n">
-        <v>50740</v>
+      <c r="C9" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B10" s="2" t="n">
         <v>44570</v>
       </c>
-      <c r="B10" t="n">
+      <c r="C10" t="n">
         <v>32032</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B11" s="2" t="n">
         <v>44571</v>
       </c>
-      <c r="B11" t="n">
+      <c r="C11" t="n">
         <v>16675</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B12" s="2" t="n">
         <v>44572</v>
       </c>
-      <c r="B12" t="n">
+      <c r="C12" t="n">
         <v>12812</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B13" s="2" t="n">
         <v>44573</v>
       </c>
-      <c r="B13" t="n">
+      <c r="C13" t="n">
         <v>13137</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B14" s="2" t="n">
         <v>44574</v>
       </c>
-      <c r="B14" t="n">
+      <c r="C14" t="n">
         <v>22843</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B15" s="2" t="n">
         <v>44575</v>
       </c>
-      <c r="B15" t="n">
+      <c r="C15" t="n">
         <v>28641</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B16" s="2" t="n">
         <v>44576</v>
       </c>
-      <c r="B16" t="n">
+      <c r="C16" t="n">
         <v>28210</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B17" s="2" t="n">
         <v>44577</v>
       </c>
-      <c r="B17" t="n">
+      <c r="C17" t="n">
         <v>19522</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B18" s="2" t="n">
         <v>44578</v>
       </c>
-      <c r="B18" t="n">
+      <c r="C18" t="n">
         <v>13446</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B19" s="2" t="n">
         <v>44579</v>
       </c>
-      <c r="B19" t="n">
+      <c r="C19" t="n">
         <v>12957</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B20" s="2" t="n">
         <v>44580</v>
       </c>
-      <c r="B20" t="n">
+      <c r="C20" t="n">
         <v>24893</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B21" s="2" t="n">
         <v>44581</v>
       </c>
-      <c r="B21" t="n">
+      <c r="C21" t="n">
         <v>32851</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B22" s="2" t="n">
         <v>44582</v>
       </c>
-      <c r="B22" t="n">
+      <c r="C22" t="n">
         <v>19021</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B23" s="2" t="n">
         <v>44583</v>
       </c>
-      <c r="B23" t="n">
+      <c r="C23" t="n">
         <v>12652</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B24" s="2" t="n">
         <v>44584</v>
       </c>
-      <c r="B24" t="n">
+      <c r="C24" t="n">
         <v>15312</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B25" s="2" t="n">
         <v>44585</v>
       </c>
-      <c r="B25" t="n">
+      <c r="C25" t="n">
         <v>23637</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B26" s="2" t="n">
         <v>44586</v>
       </c>
-      <c r="B26" t="n">
+      <c r="C26" t="n">
         <v>30964</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B27" s="2" t="n">
         <v>44587</v>
       </c>
-      <c r="B27" t="n">
+      <c r="C27" t="n">
         <v>29364</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B28" s="2" t="n">
         <v>44588</v>
       </c>
-      <c r="B28" t="n">
+      <c r="C28" t="n">
         <v>28140</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B29" s="2" t="n">
         <v>44589</v>
       </c>
-      <c r="B29" t="n">
+      <c r="C29" t="n">
         <v>25699</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B30" s="2" t="n">
         <v>44590</v>
       </c>
-      <c r="B30" t="n">
+      <c r="C30" t="n">
         <v>16844</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B31" s="2" t="n">
         <v>44591</v>
       </c>
-      <c r="B31" t="n">
+      <c r="C31" t="n">
         <v>13350</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B32" s="2" t="n">
         <v>44592</v>
       </c>
-      <c r="B32" t="n">
+      <c r="C32" t="n">
         <v>13166</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B33" s="2" t="n">
         <v>44593</v>
       </c>
-      <c r="B33" t="n">
+      <c r="C33" t="n">
         <v>26565</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B34" s="2" t="n">
         <v>44594</v>
       </c>
-      <c r="B34" t="n">
+      <c r="C34" t="n">
         <v>35099</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B35" s="2" t="n">
         <v>44595</v>
       </c>
-      <c r="B35" t="n">
+      <c r="C35" t="n">
         <v>35421</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B36" s="2" t="n">
         <v>44596</v>
       </c>
-      <c r="B36" t="n">
+      <c r="C36" t="n">
         <v>21280</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B37" s="2" t="n">
         <v>44597</v>
       </c>
-      <c r="B37" t="n">
+      <c r="C37" t="n">
         <v>12848</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B38" s="2" t="n">
         <v>44598</v>
       </c>
-      <c r="B38" t="n">
+      <c r="C38" t="n">
         <v>12356</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B39" s="2" t="n">
         <v>44599</v>
       </c>
-      <c r="B39" t="n">
+      <c r="C39" t="n">
         <v>24424</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B40" s="2" t="n">
         <v>44600</v>
       </c>
-      <c r="B40" t="n">
+      <c r="C40" t="n">
         <v>32299</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B41" s="2" t="n">
         <v>44601</v>
       </c>
-      <c r="B41" t="n">
+      <c r="C41" t="n">
         <v>31556</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B42" s="2" t="n">
         <v>44602</v>
       </c>
-      <c r="B42" t="n">
+      <c r="C42" t="n">
         <v>18220</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B43" s="2" t="n">
         <v>44603</v>
       </c>
-      <c r="B43" t="n">
+      <c r="C43" t="n">
         <v>12601</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B44" s="2" t="n">
         <v>44604</v>
       </c>
-      <c r="B44" t="n">
+      <c r="C44" t="n">
         <v>12846</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B45" s="2" t="n">
         <v>44605</v>
       </c>
-      <c r="B45" t="n">
+      <c r="C45" t="n">
         <v>28262</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B46" s="2" t="n">
         <v>44606</v>
       </c>
-      <c r="B46" t="n">
+      <c r="C46" t="n">
         <v>41905</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B47" s="2" t="n">
         <v>44607</v>
       </c>
-      <c r="B47" t="n">
+      <c r="C47" t="n">
         <v>38763</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B48" s="2" t="n">
         <v>44608</v>
       </c>
-      <c r="B48" t="n">
+      <c r="C48" t="n">
         <v>20255</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B49" s="2" t="n">
         <v>44609</v>
       </c>
-      <c r="B49" t="n">
+      <c r="C49" t="n">
         <v>12564</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B50" s="2" t="n">
         <v>44610</v>
       </c>
-      <c r="B50" t="n">
+      <c r="C50" t="n">
         <v>12687</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B51" s="2" t="n">
         <v>44611</v>
       </c>
-      <c r="B51" t="n">
+      <c r="C51" t="n">
         <v>14465</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B52" s="2" t="n">
         <v>44612</v>
       </c>
-      <c r="B52" t="n">
+      <c r="C52" t="n">
         <v>17310</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B53" s="2" t="n">
         <v>44613</v>
       </c>
-      <c r="B53" t="n">
+      <c r="C53" t="n">
         <v>17363</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B54" s="2" t="n">
         <v>44614</v>
       </c>
-      <c r="B54" t="n">
+      <c r="C54" t="n">
         <v>23593</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B55" s="2" t="n">
         <v>44615</v>
       </c>
-      <c r="B55" t="n">
+      <c r="C55" t="n">
         <v>25839</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B56" s="2" t="n">
         <v>44616</v>
       </c>
-      <c r="B56" t="n">
+      <c r="C56" t="n">
         <v>26255</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B57" s="2" t="n">
         <v>44617</v>
       </c>
-      <c r="B57" t="n">
+      <c r="C57" t="n">
         <v>18814</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B58" s="2" t="n">
         <v>44618</v>
       </c>
-      <c r="B58" t="n">
+      <c r="C58" t="n">
         <v>14600</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B59" s="2" t="n">
         <v>44619</v>
       </c>
-      <c r="B59" t="n">
+      <c r="C59" t="n">
         <v>14774</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B60" s="2" t="n">
         <v>44620</v>
       </c>
-      <c r="B60" t="n">
+      <c r="C60" t="n">
         <v>22221</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" t="n">
+        <v>1010202</v>
+      </c>
+      <c r="B61" s="2" t="n">
         <v>44621</v>
       </c>
-      <c r="B61" t="n">
+      <c r="C61" t="n">
         <v>45522</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>44562</v>
+      </c>
+      <c r="C62" t="n">
+        <v>46864</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B63" s="2" t="n">
+        <v>44563</v>
+      </c>
+      <c r="C63" t="n">
+        <v>57928</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>44564</v>
+      </c>
+      <c r="C64" t="n">
+        <v>61178</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B65" s="2" t="n">
+        <v>44565</v>
+      </c>
+      <c r="C65" t="n">
+        <v>38528</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>44566</v>
+      </c>
+      <c r="C66" t="n">
+        <v>26262</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B67" s="2" t="n">
+        <v>44567</v>
+      </c>
+      <c r="C67" t="n">
+        <v>26886</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B68" s="2" t="n">
+        <v>44568</v>
+      </c>
+      <c r="C68" t="n">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>44569</v>
+      </c>
+      <c r="C69" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>44570</v>
+      </c>
+      <c r="C70" t="n">
+        <v>64064</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>44571</v>
+      </c>
+      <c r="C71" t="n">
+        <v>33350</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>44572</v>
+      </c>
+      <c r="C72" t="n">
+        <v>25624</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B73" s="2" t="n">
+        <v>44573</v>
+      </c>
+      <c r="C73" t="n">
+        <v>26274</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>44574</v>
+      </c>
+      <c r="C74" t="n">
+        <v>45686</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B75" s="2" t="n">
+        <v>44575</v>
+      </c>
+      <c r="C75" t="n">
+        <v>57282</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>44576</v>
+      </c>
+      <c r="C76" t="n">
+        <v>56420</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>44577</v>
+      </c>
+      <c r="C77" t="n">
+        <v>39044</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>44578</v>
+      </c>
+      <c r="C78" t="n">
+        <v>26892</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B79" s="2" t="n">
+        <v>44579</v>
+      </c>
+      <c r="C79" t="n">
+        <v>25914</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>44580</v>
+      </c>
+      <c r="C80" t="n">
+        <v>49786</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B81" s="2" t="n">
+        <v>44581</v>
+      </c>
+      <c r="C81" t="n">
+        <v>65702</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>44582</v>
+      </c>
+      <c r="C82" t="n">
+        <v>38042</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>44583</v>
+      </c>
+      <c r="C83" t="n">
+        <v>25304</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B84" s="2" t="n">
+        <v>44584</v>
+      </c>
+      <c r="C84" t="n">
+        <v>30624</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B85" s="2" t="n">
+        <v>44585</v>
+      </c>
+      <c r="C85" t="n">
+        <v>47274</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B86" s="2" t="n">
+        <v>44586</v>
+      </c>
+      <c r="C86" t="n">
+        <v>61928</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B87" s="2" t="n">
+        <v>44587</v>
+      </c>
+      <c r="C87" t="n">
+        <v>58728</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B88" s="2" t="n">
+        <v>44588</v>
+      </c>
+      <c r="C88" t="n">
+        <v>56280</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B89" s="2" t="n">
+        <v>44589</v>
+      </c>
+      <c r="C89" t="n">
+        <v>51398</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B90" s="2" t="n">
+        <v>44590</v>
+      </c>
+      <c r="C90" t="n">
+        <v>33688</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B91" s="2" t="n">
+        <v>44591</v>
+      </c>
+      <c r="C91" t="n">
+        <v>26700</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B92" s="2" t="n">
+        <v>44592</v>
+      </c>
+      <c r="C92" t="n">
+        <v>26332</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B93" s="2" t="n">
+        <v>44593</v>
+      </c>
+      <c r="C93" t="n">
+        <v>53130</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B94" s="2" t="n">
+        <v>44594</v>
+      </c>
+      <c r="C94" t="n">
+        <v>70198</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B95" s="2" t="n">
+        <v>44595</v>
+      </c>
+      <c r="C95" t="n">
+        <v>70842</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B96" s="2" t="n">
+        <v>44596</v>
+      </c>
+      <c r="C96" t="n">
+        <v>42560</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B97" s="2" t="n">
+        <v>44597</v>
+      </c>
+      <c r="C97" t="n">
+        <v>25696</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B98" s="2" t="n">
+        <v>44598</v>
+      </c>
+      <c r="C98" t="n">
+        <v>24712</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B99" s="2" t="n">
+        <v>44599</v>
+      </c>
+      <c r="C99" t="n">
+        <v>48848</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B100" s="2" t="n">
+        <v>44600</v>
+      </c>
+      <c r="C100" t="n">
+        <v>64598</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B101" s="2" t="n">
+        <v>44601</v>
+      </c>
+      <c r="C101" t="n">
+        <v>63112</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B102" s="2" t="n">
+        <v>44602</v>
+      </c>
+      <c r="C102" t="n">
+        <v>36440</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B103" s="2" t="n">
+        <v>44603</v>
+      </c>
+      <c r="C103" t="n">
+        <v>25202</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B104" s="2" t="n">
+        <v>44604</v>
+      </c>
+      <c r="C104" t="n">
+        <v>25692</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B105" s="2" t="n">
+        <v>44605</v>
+      </c>
+      <c r="C105" t="n">
+        <v>56524</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B106" s="2" t="n">
+        <v>44606</v>
+      </c>
+      <c r="C106" t="n">
+        <v>83810</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B107" s="2" t="n">
+        <v>44607</v>
+      </c>
+      <c r="C107" t="n">
+        <v>77526</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B108" s="2" t="n">
+        <v>44608</v>
+      </c>
+      <c r="C108" t="n">
+        <v>40510</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B109" s="2" t="n">
+        <v>44609</v>
+      </c>
+      <c r="C109" t="n">
+        <v>25128</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B110" s="2" t="n">
+        <v>44610</v>
+      </c>
+      <c r="C110" t="n">
+        <v>25374</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B111" s="2" t="n">
+        <v>44611</v>
+      </c>
+      <c r="C111" t="n">
+        <v>28930</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B112" s="2" t="n">
+        <v>44612</v>
+      </c>
+      <c r="C112" t="n">
+        <v>34620</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B113" s="2" t="n">
+        <v>44613</v>
+      </c>
+      <c r="C113" t="n">
+        <v>34726</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B114" s="2" t="n">
+        <v>44614</v>
+      </c>
+      <c r="C114" t="n">
+        <v>47186</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B115" s="2" t="n">
+        <v>44615</v>
+      </c>
+      <c r="C115" t="n">
+        <v>51678</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B116" s="2" t="n">
+        <v>44616</v>
+      </c>
+      <c r="C116" t="n">
+        <v>52510</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B117" s="2" t="n">
+        <v>44617</v>
+      </c>
+      <c r="C117" t="n">
+        <v>37628</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B118" s="2" t="n">
+        <v>44618</v>
+      </c>
+      <c r="C118" t="n">
+        <v>29200</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B119" s="2" t="n">
+        <v>44619</v>
+      </c>
+      <c r="C119" t="n">
+        <v>29548</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B120" s="2" t="n">
+        <v>44620</v>
+      </c>
+      <c r="C120" t="n">
+        <v>44442</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>1010400</v>
+      </c>
+      <c r="B121" s="2" t="n">
+        <v>44621</v>
+      </c>
+      <c r="C121" t="n">
+        <v>91044</v>
       </c>
     </row>
   </sheetData>

</xml_diff>